<commit_message>
Aggiornamento automatico del sito — 02/08/2026 09:49
</commit_message>
<xml_diff>
--- a/data/organizzazioni.xlsx
+++ b/data/organizzazioni.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C81CD1C6-3031-468B-9EE7-080D146B986D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684519C1-BB31-45FF-8136-48F53557B87E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4212" yWindow="1944" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="38">
   <si>
     <t>Casa editrice in lingue estere</t>
   </si>
@@ -133,6 +133,12 @@
   </si>
   <si>
     <t>Partito Comunista (marxista-leninista) Italiano</t>
+  </si>
+  <si>
+    <t>Partito Comunista Unificato d'Italia</t>
+  </si>
+  <si>
+    <t>???</t>
   </si>
 </sst>
 </file>
@@ -202,12 +208,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -505,7 +510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49.44140625" customWidth="1"/>
@@ -549,7 +554,7 @@
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
       <c r="C3">
@@ -682,7 +687,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
+      <c r="A14" t="s">
         <v>4</v>
       </c>
       <c r="B14" t="s">
@@ -699,7 +704,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" t="s">
         <v>6</v>
       </c>
       <c r="B15" t="s">
@@ -797,6 +802,20 @@
       </c>
       <c r="D21">
         <v>1969</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22">
+        <v>1977</v>
+      </c>
+      <c r="D22" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>